<commit_message>
docs: versión 1.6 ajuste metodológico
Se incorpora el seguimiento de la ejecución del proyecto, el ajuste metodológico aplicado durante el Sprint 2, la actualización del backlog, los requerimientos funcionales y las nuevas tareas derivadas del cambio identificado durante el desarrollo.
</commit_message>
<xml_diff>
--- a/doc/Analisis_Requerimientos_Reservas_MesaFlow.xlsx
+++ b/doc/Analisis_Requerimientos_Reservas_MesaFlow.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Seminario Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6AEC3A-7F6D-43B2-AE63-3FE4AA1D70AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67E1FAA-54F3-42CC-BC72-0FBEC1047862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{C654E54C-59C2-4098-BDE4-CD4E1CD6717D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C654E54C-59C2-4098-BDE4-CD4E1CD6717D}"/>
   </bookViews>
   <sheets>
     <sheet name="RF" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>Reservas</t>
   </si>
   <si>
-    <t>Permite consultar disponibilidad actual y futura de un establecimiento para realizar reservas.</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
@@ -95,24 +92,15 @@
     <t>RF-010, RF-011</t>
   </si>
   <si>
-    <t>Utiliza información de mesas, reservas existentes y ocupación del establecimiento.</t>
-  </si>
-  <si>
     <t>RF-013</t>
   </si>
   <si>
     <t>Registro de reserva</t>
   </si>
   <si>
-    <t>Permite registrar reservas indicando fecha, horario, cantidad de personas y observaciones opcionales.</t>
-  </si>
-  <si>
     <t>Highest</t>
   </si>
   <si>
-    <t>Confirmación automática si existe disponibilidad clara; caso contrario queda pendiente de validación administrativa. (Decide el bar como se realizaran las reserva parametrizacion previa)</t>
-  </si>
-  <si>
     <t>RF-014</t>
   </si>
   <si>
@@ -146,9 +134,6 @@
     <t>Gestión administrativa de reservas</t>
   </si>
   <si>
-    <t>Permite administrar las reservas del establecimiento desde el panel administrativo.</t>
-  </si>
-  <si>
     <t>Web Admin</t>
   </si>
   <si>
@@ -176,9 +161,6 @@
     <t>Como cliente, quiero consultar disponibilidad y realizar una reserva para asegurar mi lugar en el establecimiento.</t>
   </si>
   <si>
-    <t>El cliente puede consultar disponibilidad actual y futura.El sistema informa mesas y capacidad disponible.El cliente puede seleccionar fecha y horario.El cliente puede indicar cantidad de personas.El sistema registra correctamente la reserva.La reserva queda confirmada o pendiente según las reglas del establecimiento.</t>
-  </si>
-  <si>
     <t>RF-012, RF-013</t>
   </si>
   <si>
@@ -200,9 +182,6 @@
     <t>Como administrador, quiero gestionar las reservas del establecimiento para controlar la disponibilidad y organización de las mesas.</t>
   </si>
   <si>
-    <t>El administrador puede visualizar reservas registradas.El administrador puede confirmar reservas pendientes.El administrador puede rechazar reservas.El administrador puede modificar reservas.El administrador puede cancelar reservas.El administrador puede consultar el historial de reservas.</t>
-  </si>
-  <si>
     <t>Actor principal</t>
   </si>
   <si>
@@ -297,6 +276,27 @@
   </si>
   <si>
     <t>ASIGANADO</t>
+  </si>
+  <si>
+    <t>Utiliza la disponibilidad de mesas individuales o agrupadas, las reservas existentes y la ocupación del establecimiento para determinar la disponibilidad de reserva.</t>
+  </si>
+  <si>
+    <t>Permite consultar la disponibilidad actual y futura de un establecimiento considerando la asignación dinámica de mesas según la cantidad de comensales.</t>
+  </si>
+  <si>
+    <t>El sistema asigna automáticamente una o varias mesas según la disponibilidad existente y las reglas configuradas para el establecimiento.</t>
+  </si>
+  <si>
+    <t>Confirmación automática si existe disponibilidad suficiente considerando la asignación dinámica de mesas; caso contrario la reserva queda pendiente de validación administrativa según la configuración del establecimiento.</t>
+  </si>
+  <si>
+    <t>Permite administrar las reservas del establecimiento desde el panel administrativo. El administrador puede consultar la asignación de mesas realizada para cada reserva.</t>
+  </si>
+  <si>
+    <t>El cliente puede consultar disponibilidad actual y futura.El sistema informa la disponibilidad considerando mesas individuales o agrupadas según la cantidad de personas..El cliente puede seleccionar fecha y horario.El cliente puede indicar cantidad de personas.El sistema registra la reserva asignando automáticamente una o varias mesas según disponibilidad.</t>
+  </si>
+  <si>
+    <t>El administrador puede visualizar reservas registradas.El administrador puede confirmar reservas pendientes.El administrador puede rechazar reservas.El administrador puede modificar reservas.El administrador puede cancelar reservas.El administrador puede consultar el historial de reservas. El administrador puede visualizar la asignación de mesas correspondiente a cada reserva.</t>
   </si>
 </sst>
 </file>
@@ -1134,6 +1134,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.33203125" customWidth="1"/>
     <col min="8" max="8" width="15.44140625" customWidth="1"/>
     <col min="9" max="9" width="13.5546875" customWidth="1"/>
@@ -1181,138 +1182,138 @@
         <v>11</v>
       </c>
       <c r="E3" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>16</v>
-      </c>
       <c r="J3" s="11" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="28.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="2:10" ht="28.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="I5" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="2:10" ht="28.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="28.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1337,13 +1338,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>2</v>
@@ -1352,76 +1353,76 @@
         <v>4</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="52.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="12" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1444,7 +1445,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:11" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="21" t="s">
         <v>0</v>
       </c>
@@ -1455,121 +1456,121 @@
         <v>2</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F2" s="22" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="28.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="8" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>9</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:11" ht="28.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="28.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="12" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K5" s="20" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1592,22 +1593,22 @@
     <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="24" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="2:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1615,19 +1616,19 @@
         <v>4</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1635,19 +1636,19 @@
         <v>5</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="32" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F4" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="34" t="s">
         <v>70</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>